<commit_message>
Add SEO language accounts to link tracking
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019u5Ro2qWzHvebyWswWY4qc
</commit_message>
<xml_diff>
--- a/Marketing/conversion-tracking/sheet/conversion-tracker.xlsx
+++ b/Marketing/conversion-tracking/sheet/conversion-tracker.xlsx
@@ -543,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -904,8 +904,56 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>seo</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SEO blog articles on salahalarm.com (one account per language)</t>
+        </is>
+      </c>
+      <c r="C8">
+        <f>COUNTIF(Videos!$C:$C,A8)</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>SUMIF(Videos!$C:$C,A8,Videos!$F:$F)</f>
+        <v/>
+      </c>
+      <c r="E8" s="3">
+        <f>SUMIF(Videos!$C:$C,A8,Videos!$L:$L)</f>
+        <v/>
+      </c>
+      <c r="F8" s="3">
+        <f>SUMIF(Videos!$C:$C,A8,Videos!$M:$M)</f>
+        <v/>
+      </c>
+      <c r="G8" s="3">
+        <f>SUMIF(Videos!$C:$C,A8,Videos!$N:$N)</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>IF(D8=0,"",E8/D8*1000)</f>
+        <v/>
+      </c>
+      <c r="I8" s="4">
+        <f>IF(D8=0,"",F8/D8*10000)</f>
+        <v/>
+      </c>
+      <c r="J8" s="4">
+        <f>IF(D8=0,"",G8/D8*10000)</f>
+        <v/>
+      </c>
+      <c r="K8" s="5">
+        <f>IF(C8=0,"",D8/C8)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I7">
+  <conditionalFormatting sqref="I2:I8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -915,7 +963,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J7">
+  <conditionalFormatting sqref="J2:J8">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -935,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1293,6 +1341,141 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>https://salahalarm.com/go/tt10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>seo-en</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>salahalarm.com/blog/en/</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>seo</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://salahalarm.com/go/seo-en</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>seo-ar</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>salahalarm.com/blog/ar/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>seo</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://salahalarm.com/go/seo-ar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>seo-tr</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>salahalarm.com/blog/tr/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>seo</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://salahalarm.com/go/seo-tr</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>seo-id</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>salahalarm.com/blog/id/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>seo</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://salahalarm.com/go/seo-id</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>seo-ur</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>salahalarm.com/blog/ur/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>seo</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://salahalarm.com/go/seo-ur</t>
         </is>
       </c>
     </row>
@@ -14324,10 +14507,10 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="B2:B401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Accounts!$A$2:$A$13</formula1>
+      <formula1>=Accounts!$A$2:$A$60</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"whatif,anim,alarm,pov,ramadan,mixed"</formula1>
+      <formula1>"whatif,anim,alarm,pov,ramadan,mixed,seo"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26894,7 +27077,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:B401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Accounts!$A$2:$A$13</formula1>
+      <formula1>=Accounts!$A$2:$A$60</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>